<commit_message>
Changed NAS excel file
</commit_message>
<xml_diff>
--- a/data/obx_xlsx/NAS.OL.xlsx
+++ b/data/obx_xlsx/NAS.OL.xlsx
@@ -12752,7 +12752,7 @@
       <c r="U56" s="15">
         <v>182.7</v>
       </c>
-      <c r="V56" s="14"/>
+      <c r="V56" s="15"/>
     </row>
     <row r="57" ht="15.0" customHeight="1">
       <c r="A57" s="16" t="s">
@@ -12761,30 +12761,84 @@
       <c r="B57" s="14">
         <v>24791.0</v>
       </c>
-      <c r="C57" s="15">
+      <c r="C57" s="17">
         <v>8490.2</v>
       </c>
-      <c r="D57" s="14"/>
-      <c r="E57" s="14"/>
-      <c r="F57" s="14"/>
-      <c r="G57" s="14"/>
-      <c r="H57" s="14"/>
-      <c r="I57" s="14"/>
-      <c r="J57" s="14"/>
-      <c r="K57" s="14"/>
-      <c r="L57" s="14"/>
-      <c r="M57" s="14"/>
-      <c r="N57" s="14"/>
-      <c r="O57" s="15">
+      <c r="D57" s="17">
+        <f t="shared" ref="D57:N57" si="1">SUM(D58,D63,D67,D71)</f>
+        <v>4878.6</v>
+      </c>
+      <c r="E57" s="17">
+        <f t="shared" si="1"/>
+        <v>4375.8</v>
+      </c>
+      <c r="F57" s="17">
+        <f t="shared" si="1"/>
+        <v>1403</v>
+      </c>
+      <c r="G57" s="17">
+        <f t="shared" si="1"/>
+        <v>6545.2</v>
+      </c>
+      <c r="H57" s="17">
+        <f t="shared" si="1"/>
+        <v>32800.2</v>
+      </c>
+      <c r="I57" s="17">
+        <f t="shared" si="1"/>
+        <v>31545</v>
+      </c>
+      <c r="J57" s="17">
+        <f t="shared" si="1"/>
+        <v>26231.8</v>
+      </c>
+      <c r="K57" s="17">
+        <f t="shared" si="1"/>
+        <v>22943.38</v>
+      </c>
+      <c r="L57" s="17">
+        <f t="shared" si="1"/>
+        <v>18872.89</v>
+      </c>
+      <c r="M57" s="17">
+        <f t="shared" si="1"/>
+        <v>12863.86</v>
+      </c>
+      <c r="N57" s="17">
+        <f t="shared" si="1"/>
+        <v>7614.65</v>
+      </c>
+      <c r="O57" s="17">
         <v>8516.7</v>
       </c>
-      <c r="P57" s="14"/>
-      <c r="Q57" s="14"/>
-      <c r="R57" s="14"/>
-      <c r="S57" s="14"/>
-      <c r="T57" s="14"/>
-      <c r="U57" s="14"/>
-      <c r="V57" s="14"/>
+      <c r="P57" s="17">
+        <f t="shared" ref="P57:V57" si="2">SUM(P56,P58,P64,P81)</f>
+        <v>3903.96</v>
+      </c>
+      <c r="Q57" s="17">
+        <f t="shared" si="2"/>
+        <v>2124.44</v>
+      </c>
+      <c r="R57" s="17">
+        <f t="shared" si="2"/>
+        <v>1009.35</v>
+      </c>
+      <c r="S57" s="17">
+        <f t="shared" si="2"/>
+        <v>558.56</v>
+      </c>
+      <c r="T57" s="17">
+        <f t="shared" si="2"/>
+        <v>238.06</v>
+      </c>
+      <c r="U57" s="17">
+        <f t="shared" si="2"/>
+        <v>152.31</v>
+      </c>
+      <c r="V57" s="17">
+        <f t="shared" si="2"/>
+        <v>1.59</v>
+      </c>
     </row>
     <row r="58" ht="15.0" customHeight="1">
       <c r="A58" s="16" t="s">
@@ -15541,9 +15595,18 @@
       <c r="H118" s="15">
         <v>4589.6</v>
       </c>
-      <c r="I118" s="14"/>
-      <c r="J118" s="14"/>
-      <c r="K118" s="14"/>
+      <c r="I118" s="17">
+        <f t="shared" ref="I118:K118" si="3">SUM(I123,I124,I125,I126)</f>
+        <v>11309.1</v>
+      </c>
+      <c r="J118" s="17">
+        <f t="shared" si="3"/>
+        <v>4244.48</v>
+      </c>
+      <c r="K118" s="17">
+        <f t="shared" si="3"/>
+        <v>4768.81</v>
+      </c>
       <c r="L118" s="15">
         <v>3041.39</v>
       </c>
@@ -15559,9 +15622,18 @@
       <c r="P118" s="15">
         <v>1551.92</v>
       </c>
-      <c r="Q118" s="14"/>
-      <c r="R118" s="14"/>
-      <c r="S118" s="14"/>
+      <c r="Q118" s="17">
+        <f t="shared" ref="Q118:S118" si="4">SUM(Q119:Q122)</f>
+        <v>520.98</v>
+      </c>
+      <c r="R118" s="17">
+        <f t="shared" si="4"/>
+        <v>675.3</v>
+      </c>
+      <c r="S118" s="17">
+        <f t="shared" si="4"/>
+        <v>257.46</v>
+      </c>
       <c r="T118" s="14"/>
       <c r="U118" s="14"/>
       <c r="V118" s="14"/>

</xml_diff>